<commit_message>
another go at it
</commit_message>
<xml_diff>
--- a/158/prob158.xlsx
+++ b/158/prob158.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
@@ -14,6 +14,12 @@
     <sheet name="seven" sheetId="4" state="visible" r:id="rId5"/>
     <sheet name="Sheet5" sheetId="5" state="visible" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="false" name="A" vbProcedure="false">Sheet5!$W$2</definedName>
+    <definedName function="false" hidden="false" name="B" vbProcedure="false">Sheet5!$W$3</definedName>
+    <definedName function="false" hidden="false" name="ll" vbProcedure="false">Sheet5!$H$3:$H$38</definedName>
+    <definedName function="false" hidden="false" name="rr" vbProcedure="false">Sheet5!$L$3:$L$38</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -24,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="35">
   <si>
     <t xml:space="preserve">a</t>
   </si>
@@ -118,6 +124,18 @@
   <si>
     <t xml:space="preserve">Minimum #'s</t>
   </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K</t>
+  </si>
 </sst>
 </file>
 
@@ -196,7 +214,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -243,6 +261,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF000000"/>
         <bgColor rgb="FF003300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -296,7 +320,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -457,6 +481,14 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -470,6 +502,30 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -3083,7 +3139,7 @@
       </c>
       <c r="G4" s="30" t="n">
         <f aca="false">0.00015+com.sun.star.sheet.addin.Analysis.getRandbetween(-10,10)/100000</f>
-        <v>0.00025</v>
+        <v>0.00023</v>
       </c>
       <c r="H4" s="30" t="s">
         <v>21</v>
@@ -3099,14 +3155,14 @@
       </c>
       <c r="E5" s="32" t="n">
         <f aca="false">E$4+com.sun.star.sheet.addin.Analysis.getRandbetween(-100,100)/1000</f>
-        <v>0.608</v>
+        <v>0.562</v>
       </c>
       <c r="F5" s="30" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="30" t="n">
         <f aca="false">0.00015+com.sun.star.sheet.addin.Analysis.getRandbetween(-10,10)/100000</f>
-        <v>0.00023</v>
+        <v>0.00013</v>
       </c>
       <c r="H5" s="30" t="s">
         <v>21</v>
@@ -3122,7 +3178,7 @@
       </c>
       <c r="E6" s="32" t="n">
         <f aca="false">E$4+com.sun.star.sheet.addin.Analysis.getRandbetween(-100,100)/1000</f>
-        <v>0.441</v>
+        <v>0.482</v>
       </c>
       <c r="F6" s="33" t="n">
         <v>5</v>
@@ -3152,7 +3208,7 @@
       </c>
       <c r="G7" s="30" t="n">
         <f aca="false">0.00015+com.sun.star.sheet.addin.Analysis.getRandbetween(-10,10)/100000</f>
-        <v>0.00014</v>
+        <v>7E-005</v>
       </c>
       <c r="H7" s="30" t="s">
         <v>21</v>
@@ -3168,14 +3224,14 @@
       </c>
       <c r="E8" s="32" t="n">
         <f aca="false">E$4+com.sun.star.sheet.addin.Analysis.getRandbetween(-100,100)/1000</f>
-        <v>0.509</v>
+        <v>0.492</v>
       </c>
       <c r="F8" s="30" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="30" t="n">
         <f aca="false">0.00015+com.sun.star.sheet.addin.Analysis.getRandbetween(-10,10)/100000</f>
-        <v>0.00012</v>
+        <v>0.00022</v>
       </c>
       <c r="H8" s="33" t="n">
         <v>-2</v>
@@ -3191,14 +3247,14 @@
       </c>
       <c r="E9" s="32" t="n">
         <f aca="false">E$4+com.sun.star.sheet.addin.Analysis.getRandbetween(-100,100)/1000</f>
-        <v>0.551</v>
+        <v>0.524</v>
       </c>
       <c r="F9" s="30" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="30" t="n">
         <f aca="false">0.00015+com.sun.star.sheet.addin.Analysis.getRandbetween(-10,10)/100000</f>
-        <v>0.00021</v>
+        <v>9E-005</v>
       </c>
       <c r="H9" s="30" t="s">
         <v>21</v>
@@ -3214,14 +3270,14 @@
       </c>
       <c r="E10" s="32" t="n">
         <f aca="false">E$4+com.sun.star.sheet.addin.Analysis.getRandbetween(-100,100)/1000</f>
-        <v>0.492</v>
+        <v>0.61</v>
       </c>
       <c r="F10" s="30" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="30" t="n">
         <f aca="false">0.00015+com.sun.star.sheet.addin.Analysis.getRandbetween(-10,10)/100000</f>
-        <v>9E-005</v>
+        <v>0.00013</v>
       </c>
       <c r="H10" s="30" t="s">
         <v>21</v>
@@ -3237,14 +3293,14 @@
       </c>
       <c r="E11" s="32" t="n">
         <f aca="false">E$4+com.sun.star.sheet.addin.Analysis.getRandbetween(-100,100)/1000</f>
-        <v>0.445</v>
+        <v>0.571</v>
       </c>
       <c r="F11" s="30" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="30" t="n">
         <f aca="false">0.00015+com.sun.star.sheet.addin.Analysis.getRandbetween(-10,10)/100000</f>
-        <v>0.00016</v>
+        <v>8E-005</v>
       </c>
       <c r="H11" s="30" t="s">
         <v>21</v>
@@ -3276,7 +3332,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q58"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="11.79"/>
@@ -5271,21 +5327,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AK54"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="4" style="0" width="4.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="5.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="5.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="1.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="18" style="0" width="5.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="26" style="0" width="6.94"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="23" t="n">
-        <v>19</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>30</v>
-      </c>
+      <c r="A1" s="23"/>
+      <c r="B1" s="1"/>
       <c r="C1" s="23"/>
       <c r="D1" s="38"/>
       <c r="E1" s="39"/>
@@ -5293,93 +5348,189 @@
       <c r="G1" s="39"/>
       <c r="H1" s="38"/>
       <c r="I1" s="39"/>
-      <c r="J1" s="38" t="n">
-        <v>7</v>
-      </c>
-      <c r="K1" s="39" t="n">
-        <v>1</v>
-      </c>
+      <c r="J1" s="38"/>
+      <c r="K1" s="39"/>
       <c r="L1" s="38"/>
       <c r="M1" s="39"/>
       <c r="N1" s="23"/>
       <c r="O1" s="23"/>
       <c r="P1" s="23"/>
       <c r="Q1" s="23"/>
+      <c r="Z1" s="0" t="n">
+        <f aca="false">COMBIN(AA1,AB1)</f>
+        <v>190</v>
+      </c>
+      <c r="AA1" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB1" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC1" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD1" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE1" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF1" s="40"/>
+      <c r="AG1" s="40"/>
+      <c r="AH1" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ1" s="0" t="n">
+        <f aca="false">Z1*AH1</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
+      <c r="A2" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
       <c r="C2" s="23"/>
-      <c r="D2" s="39"/>
+      <c r="D2" s="38"/>
       <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
+      <c r="F2" s="38"/>
       <c r="G2" s="39"/>
-      <c r="H2" s="39" t="n">
-        <v>6</v>
-      </c>
+      <c r="H2" s="38"/>
       <c r="I2" s="39"/>
-      <c r="J2" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="39"/>
-      <c r="L2" s="39" t="n">
-        <v>6</v>
-      </c>
+      <c r="J2" s="38" t="n">
+        <v>7</v>
+      </c>
+      <c r="K2" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="38"/>
       <c r="M2" s="39"/>
       <c r="N2" s="23"/>
       <c r="O2" s="23"/>
       <c r="P2" s="23"/>
       <c r="Q2" s="23"/>
+      <c r="V2" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="W2" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z2" s="0" t="n">
+        <f aca="false">COMBIN(AA2,AB2)</f>
+        <v>190</v>
+      </c>
+      <c r="AA2" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB2" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD2" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE2" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF2" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG2" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH2" s="0" t="n">
+        <f aca="false">COMBIN(AF2,AG2)</f>
+        <v>3</v>
+      </c>
+      <c r="AJ2" s="0" t="n">
+        <f aca="false">Z2*AH2</f>
+        <v>570</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="B3" s="23" t="n">
-        <v>19</v>
-      </c>
-      <c r="C3" s="23" t="n">
-        <v>171</v>
-      </c>
+      <c r="A3" s="23"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
       <c r="D3" s="39"/>
       <c r="E3" s="39"/>
       <c r="F3" s="39"/>
       <c r="G3" s="39"/>
       <c r="H3" s="39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I3" s="39"/>
-      <c r="J3" s="39"/>
+      <c r="J3" s="39" t="n">
+        <v>0</v>
+      </c>
       <c r="K3" s="39"/>
       <c r="L3" s="39" t="n">
         <v>6</v>
       </c>
       <c r="M3" s="39"/>
-      <c r="N3" s="23" t="n">
-        <v>6</v>
-      </c>
+      <c r="N3" s="23"/>
       <c r="O3" s="23"/>
-      <c r="P3" s="23" t="n">
-        <v>1026</v>
-      </c>
+      <c r="P3" s="23"/>
       <c r="Q3" s="23"/>
+      <c r="V3" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="W3" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z3" s="0" t="n">
+        <f aca="false">COMBIN(AA3,AB3)</f>
+        <v>190</v>
+      </c>
+      <c r="AA3" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB3" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD3" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE3" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF3" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG3" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH3" s="0" t="n">
+        <f aca="false">COMBIN(AF3,AG3)</f>
+        <v>3</v>
+      </c>
+      <c r="AJ3" s="0" t="n">
+        <f aca="false">Z3*AH3</f>
+        <v>570</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" s="23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4" s="23" t="n">
-        <v>190</v>
+        <v>171</v>
       </c>
       <c r="D4" s="39"/>
       <c r="E4" s="39"/>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
       <c r="H4" s="39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I4" s="39"/>
       <c r="J4" s="39"/>
@@ -5393,26 +5544,59 @@
       </c>
       <c r="O4" s="23"/>
       <c r="P4" s="23" t="n">
+        <v>1026</v>
+      </c>
+      <c r="Q4" s="23"/>
+      <c r="Z4" s="0" t="n">
+        <f aca="false">COMBIN(AA4,AB4)</f>
+        <v>190</v>
+      </c>
+      <c r="AA4" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB4" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD4" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE4" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF4" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG4" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH4" s="0" t="n">
+        <f aca="false">COMBIN(AF4,AG4)</f>
+        <v>6</v>
+      </c>
+      <c r="AJ4" s="0" t="n">
+        <f aca="false">Z4*AH4</f>
         <v>1140</v>
       </c>
-      <c r="Q4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" s="23" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="23" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="D5" s="39"/>
       <c r="E5" s="39"/>
       <c r="F5" s="39"/>
       <c r="G5" s="39"/>
       <c r="H5" s="39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I5" s="39"/>
       <c r="J5" s="39"/>
@@ -5426,26 +5610,54 @@
       </c>
       <c r="O5" s="23"/>
       <c r="P5" s="23" t="n">
-        <v>1260</v>
+        <v>1140</v>
       </c>
       <c r="Q5" s="23"/>
+      <c r="Z5" s="0" t="n">
+        <f aca="false">COMBIN(AA5,AB5)</f>
+        <v>190</v>
+      </c>
+      <c r="AA5" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB5" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC5" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD5" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE5" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF5" s="40"/>
+      <c r="AG5" s="40"/>
+      <c r="AH5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" s="0" t="n">
+        <f aca="false">Z5*AH5</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" s="23" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>231</v>
+        <v>210</v>
       </c>
       <c r="D6" s="39"/>
       <c r="E6" s="39"/>
       <c r="F6" s="39"/>
       <c r="G6" s="39"/>
       <c r="H6" s="39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" s="39"/>
       <c r="J6" s="39"/>
@@ -5459,9 +5671,42 @@
       </c>
       <c r="O6" s="23"/>
       <c r="P6" s="23" t="n">
-        <v>1386</v>
+        <v>1260</v>
       </c>
       <c r="Q6" s="23"/>
+      <c r="Z6" s="0" t="n">
+        <f aca="false">COMBIN(AA6,AB6)</f>
+        <v>190</v>
+      </c>
+      <c r="AA6" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB6" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC6" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD6" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE6" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF6" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG6" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH6" s="0" t="n">
+        <f aca="false">COMBIN(AF6,AG6)</f>
+        <v>1</v>
+      </c>
+      <c r="AJ6" s="0" t="n">
+        <f aca="false">Z6*AH6</f>
+        <v>190</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="n">
@@ -5470,15 +5715,15 @@
       <c r="B7" s="23" t="n">
         <v>22</v>
       </c>
-      <c r="C7" s="23" t="n">
-        <v>231</v>
+      <c r="C7" s="23" t="s">
+        <v>33</v>
       </c>
       <c r="D7" s="39"/>
       <c r="E7" s="39"/>
       <c r="F7" s="39"/>
       <c r="G7" s="39"/>
       <c r="H7" s="39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" s="39"/>
       <c r="J7" s="39"/>
@@ -5495,29 +5740,62 @@
         <v>1386</v>
       </c>
       <c r="Q7" s="23"/>
+      <c r="Z7" s="0" t="n">
+        <f aca="false">COMBIN(AA7,AB7)</f>
+        <v>190</v>
+      </c>
+      <c r="AA7" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB7" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC7" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD7" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE7" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF7" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG7" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH7" s="0" t="n">
+        <f aca="false">COMBIN(AF7,AG7)</f>
+        <v>3</v>
+      </c>
+      <c r="AJ7" s="0" t="n">
+        <f aca="false">Z7*AH7</f>
+        <v>570</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B8" s="23" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C8" s="23" t="n">
-        <v>171</v>
+        <v>231</v>
       </c>
       <c r="D8" s="39"/>
       <c r="E8" s="39"/>
       <c r="F8" s="39"/>
       <c r="G8" s="39"/>
       <c r="H8" s="39" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I8" s="39"/>
       <c r="J8" s="39"/>
       <c r="K8" s="39"/>
       <c r="L8" s="39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M8" s="39"/>
       <c r="N8" s="23" t="n">
@@ -5525,12 +5803,47 @@
       </c>
       <c r="O8" s="23"/>
       <c r="P8" s="23" t="n">
+        <v>1386</v>
+      </c>
+      <c r="Q8" s="23"/>
+      <c r="Z8" s="0" t="n">
+        <f aca="false">COMBIN(AA8,AB8)</f>
+        <v>171</v>
+      </c>
+      <c r="AA8" s="40" t="n">
+        <v>19</v>
+      </c>
+      <c r="AB8" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC8" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE8" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF8" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG8" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH8" s="0" t="n">
+        <f aca="false">COMBIN(AF8,AG8)</f>
+        <v>6</v>
+      </c>
+      <c r="AJ8" s="0" t="n">
+        <f aca="false">Z8*AH8</f>
         <v>1026</v>
       </c>
-      <c r="Q8" s="23"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23"/>
+      <c r="A9" s="23" t="n">
+        <v>0</v>
+      </c>
       <c r="B9" s="23" t="n">
         <v>19</v>
       </c>
@@ -5542,75 +5855,139 @@
       <c r="F9" s="39"/>
       <c r="G9" s="39"/>
       <c r="H9" s="39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I9" s="39"/>
-      <c r="J9" s="39" t="n">
-        <v>0</v>
-      </c>
+      <c r="J9" s="39"/>
       <c r="K9" s="39"/>
       <c r="L9" s="39" t="n">
         <v>5</v>
       </c>
       <c r="M9" s="39"/>
       <c r="N9" s="23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O9" s="23"/>
       <c r="P9" s="23" t="n">
-        <v>0</v>
+        <v>1026</v>
       </c>
       <c r="Q9" s="23"/>
+      <c r="Z9" s="0" t="n">
+        <f aca="false">COMBIN(AA9,AB9)</f>
+        <v>190</v>
+      </c>
+      <c r="AA9" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB9" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC9" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD9" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE9" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF9" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG9" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH9" s="0" t="n">
+        <f aca="false">COMBIN(AF9,AG9)</f>
+        <v>1</v>
+      </c>
+      <c r="AJ9" s="0" t="n">
+        <f aca="false">Z9*AH9</f>
+        <v>190</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="n">
-        <v>1</v>
-      </c>
+      <c r="A10" s="23"/>
       <c r="B10" s="23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C10" s="23" t="n">
-        <v>190</v>
+        <v>171</v>
       </c>
       <c r="D10" s="39"/>
       <c r="E10" s="39"/>
       <c r="F10" s="39"/>
       <c r="G10" s="39"/>
       <c r="H10" s="39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I10" s="39"/>
-      <c r="J10" s="39"/>
+      <c r="J10" s="39" t="n">
+        <v>0</v>
+      </c>
       <c r="K10" s="39"/>
       <c r="L10" s="39" t="n">
         <v>5</v>
       </c>
       <c r="M10" s="39"/>
       <c r="N10" s="23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O10" s="23"/>
       <c r="P10" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="23"/>
+      <c r="Z10" s="0" t="n">
+        <f aca="false">COMBIN(AA10,AB10)</f>
+        <v>190</v>
+      </c>
+      <c r="AA10" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB10" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC10" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD10" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE10" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF10" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG10" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH10" s="0" t="n">
+        <f aca="false">COMBIN(AF10,AG10)</f>
+        <v>3</v>
+      </c>
+      <c r="AJ10" s="0" t="n">
+        <f aca="false">Z10*AH10</f>
         <v>570</v>
       </c>
-      <c r="Q10" s="23"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" s="23" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C11" s="23" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="D11" s="39"/>
       <c r="E11" s="39"/>
       <c r="F11" s="39"/>
       <c r="G11" s="39"/>
       <c r="H11" s="39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I11" s="39"/>
       <c r="J11" s="39"/>
@@ -5624,26 +6001,59 @@
       </c>
       <c r="O11" s="23"/>
       <c r="P11" s="23" t="n">
-        <v>630</v>
+        <v>570</v>
       </c>
       <c r="Q11" s="23"/>
+      <c r="Z11" s="0" t="n">
+        <f aca="false">COMBIN(AA11,AB11)</f>
+        <v>153</v>
+      </c>
+      <c r="AA11" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="AB11" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC11" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD11" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE11" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF11" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG11" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH11" s="0" t="n">
+        <f aca="false">COMBIN(AF11,AG11)</f>
+        <v>6</v>
+      </c>
+      <c r="AJ11" s="0" t="n">
+        <f aca="false">Z11*AH11</f>
+        <v>918</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B12" s="23" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C12" s="23" t="n">
-        <v>231</v>
+        <v>210</v>
       </c>
       <c r="D12" s="39"/>
       <c r="E12" s="39"/>
       <c r="F12" s="39"/>
       <c r="G12" s="39"/>
       <c r="H12" s="39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I12" s="39"/>
       <c r="J12" s="39"/>
@@ -5657,9 +6067,38 @@
       </c>
       <c r="O12" s="23"/>
       <c r="P12" s="23" t="n">
-        <v>693</v>
+        <v>630</v>
       </c>
       <c r="Q12" s="23"/>
+      <c r="Z12" s="0" t="n">
+        <f aca="false">COMBIN(AA12,AB12)</f>
+        <v>190</v>
+      </c>
+      <c r="AA12" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB12" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC12" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD12" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE12" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF12" s="40"/>
+      <c r="AG12" s="40"/>
+      <c r="AH12" s="0" t="n">
+        <f aca="false">COMBIN(AF12,AG12)</f>
+        <v>1</v>
+      </c>
+      <c r="AJ12" s="0" t="n">
+        <f aca="false">Z12*AH12</f>
+        <v>190</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="n">
@@ -5676,7 +6115,7 @@
       <c r="F13" s="39"/>
       <c r="G13" s="39"/>
       <c r="H13" s="39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="39"/>
       <c r="J13" s="39"/>
@@ -5693,6 +6132,39 @@
         <v>693</v>
       </c>
       <c r="Q13" s="23"/>
+      <c r="Z13" s="0" t="n">
+        <f aca="false">COMBIN(AA13,AB13)</f>
+        <v>190</v>
+      </c>
+      <c r="AA13" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB13" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC13" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD13" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE13" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF13" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG13" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH13" s="0" t="n">
+        <f aca="false">COMBIN(AF13,AG13)</f>
+        <v>3</v>
+      </c>
+      <c r="AJ13" s="0" t="n">
+        <f aca="false">Z13*AH13</f>
+        <v>570</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="n">
@@ -5709,13 +6181,13 @@
       <c r="F14" s="39"/>
       <c r="G14" s="39"/>
       <c r="H14" s="39" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I14" s="39"/>
       <c r="J14" s="39"/>
       <c r="K14" s="39"/>
       <c r="L14" s="39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M14" s="39"/>
       <c r="N14" s="23" t="n">
@@ -5726,23 +6198,56 @@
         <v>693</v>
       </c>
       <c r="Q14" s="23"/>
+      <c r="Z14" s="0" t="n">
+        <f aca="false">COMBIN(AA14,AB14)</f>
+        <v>153</v>
+      </c>
+      <c r="AA14" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="AB14" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC14" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD14" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE14" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF14" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG14" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH14" s="0" t="n">
+        <f aca="false">COMBIN(AF14,AG14)</f>
+        <v>6</v>
+      </c>
+      <c r="AJ14" s="0" t="n">
+        <f aca="false">Z14*AH14</f>
+        <v>918</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B15" s="23" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C15" s="23" t="n">
-        <v>171</v>
+        <v>231</v>
       </c>
       <c r="D15" s="39"/>
       <c r="E15" s="39"/>
       <c r="F15" s="39"/>
       <c r="G15" s="39"/>
       <c r="H15" s="39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I15" s="39"/>
       <c r="J15" s="39"/>
@@ -5756,12 +6261,43 @@
       </c>
       <c r="O15" s="23"/>
       <c r="P15" s="23" t="n">
-        <v>513</v>
+        <v>693</v>
       </c>
       <c r="Q15" s="23"/>
+      <c r="Z15" s="0" t="n">
+        <f aca="false">COMBIN(AA15,AB15)</f>
+        <v>190</v>
+      </c>
+      <c r="AA15" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="AB15" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC15" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD15" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE15" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF15" s="40"/>
+      <c r="AG15" s="40"/>
+      <c r="AH15" s="0" t="n">
+        <f aca="false">COMBIN(AF15,AG15)</f>
+        <v>1</v>
+      </c>
+      <c r="AJ15" s="0" t="n">
+        <f aca="false">Z15*AH15</f>
+        <v>190</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23"/>
+      <c r="A16" s="23" t="n">
+        <v>0</v>
+      </c>
       <c r="B16" s="23" t="n">
         <v>19</v>
       </c>
@@ -5773,75 +6309,139 @@
       <c r="F16" s="39"/>
       <c r="G16" s="39"/>
       <c r="H16" s="39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I16" s="39"/>
-      <c r="J16" s="39" t="n">
-        <v>0</v>
-      </c>
+      <c r="J16" s="39"/>
       <c r="K16" s="39"/>
       <c r="L16" s="39" t="n">
         <v>4</v>
       </c>
       <c r="M16" s="39"/>
       <c r="N16" s="23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O16" s="23"/>
       <c r="P16" s="23" t="n">
-        <v>0</v>
+        <v>513</v>
       </c>
       <c r="Q16" s="23"/>
+      <c r="Z16" s="0" t="n">
+        <f aca="false">COMBIN(AA16,AB16)</f>
+        <v>171</v>
+      </c>
+      <c r="AA16" s="40" t="n">
+        <v>19</v>
+      </c>
+      <c r="AB16" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC16" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD16" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE16" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF16" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG16" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH16" s="0" t="n">
+        <f aca="false">COMBIN(AF16,AG16)</f>
+        <v>3</v>
+      </c>
+      <c r="AJ16" s="0" t="n">
+        <f aca="false">Z16*AH16</f>
+        <v>513</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="n">
-        <v>1</v>
-      </c>
+      <c r="A17" s="23"/>
       <c r="B17" s="23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C17" s="23" t="n">
-        <v>190</v>
+        <v>171</v>
       </c>
       <c r="D17" s="39"/>
       <c r="E17" s="39"/>
       <c r="F17" s="39"/>
       <c r="G17" s="39"/>
       <c r="H17" s="39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I17" s="39"/>
-      <c r="J17" s="39"/>
+      <c r="J17" s="39" t="n">
+        <v>0</v>
+      </c>
       <c r="K17" s="39"/>
       <c r="L17" s="39" t="n">
         <v>4</v>
       </c>
       <c r="M17" s="39"/>
       <c r="N17" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O17" s="23"/>
       <c r="P17" s="23" t="n">
-        <v>190</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="23"/>
+      <c r="Z17" s="0" t="n">
+        <f aca="false">COMBIN(AA17,AB17)</f>
+        <v>153</v>
+      </c>
+      <c r="AA17" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="AB17" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC17" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD17" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE17" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF17" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG17" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH17" s="0" t="n">
+        <f aca="false">COMBIN(AF17,AG17)</f>
+        <v>6</v>
+      </c>
+      <c r="AJ17" s="0" t="n">
+        <f aca="false">Z17*AH17</f>
+        <v>918</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" s="23" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C18" s="23" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="D18" s="39"/>
       <c r="E18" s="39"/>
       <c r="F18" s="39"/>
       <c r="G18" s="39"/>
       <c r="H18" s="39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I18" s="39"/>
       <c r="J18" s="39"/>
@@ -5855,26 +6455,55 @@
       </c>
       <c r="O18" s="23"/>
       <c r="P18" s="23" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="Q18" s="23"/>
+      <c r="Z18" s="0" t="n">
+        <f aca="false">COMBIN(AA18,AB18)</f>
+        <v>153</v>
+      </c>
+      <c r="AA18" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="AB18" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC18" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD18" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE18" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF18" s="40"/>
+      <c r="AG18" s="40"/>
+      <c r="AH18" s="0" t="n">
+        <f aca="false">COMBIN(AF18,AG18)</f>
+        <v>1</v>
+      </c>
+      <c r="AJ18" s="0" t="n">
+        <f aca="false">Z18*AH18</f>
+        <v>153</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B19" s="23" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C19" s="23" t="n">
-        <v>231</v>
+        <v>210</v>
       </c>
       <c r="D19" s="39"/>
       <c r="E19" s="39"/>
       <c r="F19" s="39"/>
       <c r="G19" s="39"/>
       <c r="H19" s="39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I19" s="39"/>
       <c r="J19" s="39"/>
@@ -5888,9 +6517,42 @@
       </c>
       <c r="O19" s="23"/>
       <c r="P19" s="23" t="n">
-        <v>231</v>
+        <v>210</v>
       </c>
       <c r="Q19" s="23"/>
+      <c r="Z19" s="0" t="n">
+        <f aca="false">COMBIN(AA19,AB19)</f>
+        <v>153</v>
+      </c>
+      <c r="AA19" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="AB19" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC19" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD19" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE19" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF19" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG19" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH19" s="0" t="n">
+        <f aca="false">COMBIN(AF19,AG19)</f>
+        <v>3</v>
+      </c>
+      <c r="AJ19" s="0" t="n">
+        <f aca="false">Z19*AH19</f>
+        <v>459</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="n">
@@ -5907,13 +6569,13 @@
       <c r="F20" s="39"/>
       <c r="G20" s="39"/>
       <c r="H20" s="39" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I20" s="39"/>
       <c r="J20" s="39"/>
       <c r="K20" s="39"/>
       <c r="L20" s="39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M20" s="39"/>
       <c r="N20" s="23" t="n">
@@ -5924,6 +6586,39 @@
         <v>231</v>
       </c>
       <c r="Q20" s="23"/>
+      <c r="Z20" s="0" t="n">
+        <f aca="false">COMBIN(AA20,AB20)</f>
+        <v>153</v>
+      </c>
+      <c r="AA20" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="AB20" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC20" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD20" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE20" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF20" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG20" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH20" s="0" t="n">
+        <f aca="false">COMBIN(AF20,AG20)</f>
+        <v>6</v>
+      </c>
+      <c r="AJ20" s="0" t="n">
+        <f aca="false">Z20*AH20</f>
+        <v>918</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="n">
@@ -5940,7 +6635,7 @@
       <c r="F21" s="39"/>
       <c r="G21" s="39"/>
       <c r="H21" s="39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I21" s="39"/>
       <c r="J21" s="39"/>
@@ -5957,23 +6652,36 @@
         <v>231</v>
       </c>
       <c r="Q21" s="23"/>
+      <c r="AA21" s="40"/>
+      <c r="AB21" s="40"/>
+      <c r="AC21" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD21" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE21" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF21" s="40"/>
+      <c r="AG21" s="40"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B22" s="23" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C22" s="23" t="n">
-        <v>171</v>
+        <v>231</v>
       </c>
       <c r="D22" s="39"/>
       <c r="E22" s="39"/>
       <c r="F22" s="39"/>
       <c r="G22" s="39"/>
       <c r="H22" s="39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I22" s="39"/>
       <c r="J22" s="39"/>
@@ -5987,12 +6695,28 @@
       </c>
       <c r="O22" s="23"/>
       <c r="P22" s="23" t="n">
-        <v>171</v>
+        <v>231</v>
       </c>
       <c r="Q22" s="23"/>
+      <c r="AA22" s="41"/>
+      <c r="AB22" s="41"/>
+      <c r="AC22" s="41"/>
+      <c r="AD22" s="41"/>
+      <c r="AE22" s="41"/>
+      <c r="AF22" s="41"/>
+      <c r="AG22" s="41"/>
+      <c r="AJ22" s="0" t="n">
+        <f aca="false">SUM(AJ2:AJ21)</f>
+        <v>10573</v>
+      </c>
+      <c r="AK22" s="21" t="n">
+        <v>11420</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23"/>
+      <c r="A23" s="23" t="n">
+        <v>0</v>
+      </c>
       <c r="B23" s="23" t="n">
         <v>19</v>
       </c>
@@ -6004,75 +6728,91 @@
       <c r="F23" s="39"/>
       <c r="G23" s="39"/>
       <c r="H23" s="39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I23" s="39"/>
-      <c r="J23" s="39" t="n">
-        <v>0</v>
-      </c>
+      <c r="J23" s="39"/>
       <c r="K23" s="39"/>
       <c r="L23" s="39" t="n">
         <v>3</v>
       </c>
       <c r="M23" s="39"/>
       <c r="N23" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23" s="23"/>
       <c r="P23" s="23" t="n">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="Q23" s="23"/>
+      <c r="AA23" s="41"/>
+      <c r="AB23" s="41"/>
+      <c r="AC23" s="41"/>
+      <c r="AD23" s="41"/>
+      <c r="AE23" s="41"/>
+      <c r="AF23" s="41"/>
+      <c r="AG23" s="41"/>
+      <c r="AJ23" s="0" t="n">
+        <f aca="false">AK22-AJ22</f>
+        <v>847</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="23" t="n">
-        <v>1</v>
-      </c>
+      <c r="A24" s="23"/>
       <c r="B24" s="23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C24" s="23" t="n">
-        <v>190</v>
+        <v>171</v>
       </c>
       <c r="D24" s="39"/>
       <c r="E24" s="39"/>
       <c r="F24" s="39"/>
       <c r="G24" s="39"/>
       <c r="H24" s="39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I24" s="39"/>
-      <c r="J24" s="39"/>
+      <c r="J24" s="39" t="n">
+        <v>0</v>
+      </c>
       <c r="K24" s="39"/>
       <c r="L24" s="39" t="n">
         <v>3</v>
       </c>
       <c r="M24" s="39"/>
       <c r="N24" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24" s="23"/>
       <c r="P24" s="23" t="n">
-        <v>190</v>
+        <v>0</v>
       </c>
       <c r="Q24" s="23"/>
+      <c r="AA24" s="41"/>
+      <c r="AB24" s="41"/>
+      <c r="AC24" s="41"/>
+      <c r="AD24" s="41"/>
+      <c r="AE24" s="41"/>
+      <c r="AF24" s="41"/>
+      <c r="AG24" s="41"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B25" s="23" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C25" s="23" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="D25" s="39"/>
       <c r="E25" s="39"/>
       <c r="F25" s="39"/>
       <c r="G25" s="39"/>
       <c r="H25" s="39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I25" s="39"/>
       <c r="J25" s="39"/>
@@ -6086,55 +6826,71 @@
       </c>
       <c r="O25" s="23"/>
       <c r="P25" s="23" t="n">
+        <v>190</v>
+      </c>
+      <c r="Q25" s="23"/>
+      <c r="AA25" s="41"/>
+      <c r="AB25" s="41"/>
+      <c r="AC25" s="41"/>
+      <c r="AD25" s="41"/>
+      <c r="AE25" s="41"/>
+      <c r="AF25" s="41"/>
+      <c r="AG25" s="41"/>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="C26" s="23" t="n">
         <v>210</v>
-      </c>
-      <c r="Q25" s="23"/>
-    </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="23"/>
-      <c r="B26" s="23" t="n">
-        <v>17</v>
-      </c>
-      <c r="C26" s="23" t="n">
-        <v>136</v>
       </c>
       <c r="D26" s="39"/>
       <c r="E26" s="39"/>
       <c r="F26" s="39"/>
       <c r="G26" s="39"/>
       <c r="H26" s="39" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I26" s="39"/>
       <c r="J26" s="39"/>
       <c r="K26" s="39"/>
       <c r="L26" s="39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M26" s="39"/>
       <c r="N26" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O26" s="23"/>
       <c r="P26" s="23" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="Q26" s="23"/>
+      <c r="AA26" s="41"/>
+      <c r="AB26" s="41"/>
+      <c r="AC26" s="41"/>
+      <c r="AD26" s="41"/>
+      <c r="AE26" s="41"/>
+      <c r="AF26" s="41"/>
+      <c r="AG26" s="41"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="23"/>
       <c r="B27" s="23" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C27" s="23" t="n">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="D27" s="39"/>
       <c r="E27" s="39"/>
       <c r="F27" s="39"/>
       <c r="G27" s="39"/>
       <c r="H27" s="39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I27" s="39"/>
       <c r="J27" s="39"/>
@@ -6151,21 +6907,28 @@
         <v>0</v>
       </c>
       <c r="Q27" s="23"/>
+      <c r="AA27" s="41"/>
+      <c r="AB27" s="41"/>
+      <c r="AC27" s="41"/>
+      <c r="AD27" s="41"/>
+      <c r="AE27" s="41"/>
+      <c r="AF27" s="41"/>
+      <c r="AG27" s="41"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="23"/>
       <c r="B28" s="23" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C28" s="23" t="n">
-        <v>171</v>
+        <v>153</v>
       </c>
       <c r="D28" s="39"/>
       <c r="E28" s="39"/>
       <c r="F28" s="39"/>
       <c r="G28" s="39"/>
       <c r="H28" s="39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I28" s="39"/>
       <c r="J28" s="39"/>
@@ -6186,17 +6949,17 @@
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="23"/>
       <c r="B29" s="23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C29" s="23" t="n">
-        <v>190</v>
+        <v>171</v>
       </c>
       <c r="D29" s="39"/>
       <c r="E29" s="39"/>
       <c r="F29" s="39"/>
       <c r="G29" s="39"/>
       <c r="H29" s="39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I29" s="39"/>
       <c r="J29" s="39"/>
@@ -6217,17 +6980,17 @@
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23"/>
       <c r="B30" s="23" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C30" s="23" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="D30" s="39"/>
       <c r="E30" s="39"/>
       <c r="F30" s="39"/>
       <c r="G30" s="39"/>
       <c r="H30" s="39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I30" s="39"/>
       <c r="J30" s="39"/>
@@ -6258,7 +7021,7 @@
       <c r="F31" s="39"/>
       <c r="G31" s="39"/>
       <c r="H31" s="39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I31" s="39"/>
       <c r="J31" s="39"/>
@@ -6279,23 +7042,23 @@
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23"/>
       <c r="B32" s="23" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C32" s="23" t="n">
-        <v>136</v>
+        <v>210</v>
       </c>
       <c r="D32" s="39"/>
       <c r="E32" s="39"/>
       <c r="F32" s="39"/>
       <c r="G32" s="39"/>
       <c r="H32" s="39" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I32" s="39"/>
       <c r="J32" s="39"/>
       <c r="K32" s="39"/>
       <c r="L32" s="39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M32" s="39"/>
       <c r="N32" s="23" t="n">
@@ -6310,17 +7073,17 @@
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="23"/>
       <c r="B33" s="23" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C33" s="23" t="n">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="D33" s="39"/>
       <c r="E33" s="39"/>
       <c r="F33" s="39"/>
       <c r="G33" s="39"/>
       <c r="H33" s="39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I33" s="39"/>
       <c r="J33" s="39"/>
@@ -6341,17 +7104,17 @@
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="23"/>
       <c r="B34" s="23" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C34" s="23" t="n">
-        <v>171</v>
+        <v>153</v>
       </c>
       <c r="D34" s="39"/>
       <c r="E34" s="39"/>
       <c r="F34" s="39"/>
       <c r="G34" s="39"/>
       <c r="H34" s="39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I34" s="39"/>
       <c r="J34" s="39"/>
@@ -6372,17 +7135,17 @@
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="23"/>
       <c r="B35" s="23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C35" s="23" t="n">
-        <v>190</v>
+        <v>171</v>
       </c>
       <c r="D35" s="39"/>
       <c r="E35" s="39"/>
       <c r="F35" s="39"/>
       <c r="G35" s="39"/>
       <c r="H35" s="39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I35" s="39"/>
       <c r="J35" s="39"/>
@@ -6403,17 +7166,17 @@
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="23"/>
       <c r="B36" s="23" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C36" s="23" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="D36" s="39"/>
       <c r="E36" s="39"/>
       <c r="F36" s="39"/>
       <c r="G36" s="39"/>
       <c r="H36" s="39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I36" s="39"/>
       <c r="J36" s="39"/>
@@ -6434,17 +7197,17 @@
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="23"/>
       <c r="B37" s="23" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C37" s="23" t="n">
-        <v>231</v>
+        <v>210</v>
       </c>
       <c r="D37" s="39"/>
       <c r="E37" s="39"/>
       <c r="F37" s="39"/>
       <c r="G37" s="39"/>
       <c r="H37" s="39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I37" s="39"/>
       <c r="J37" s="39"/>
@@ -6464,26 +7227,34 @@
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="23"/>
-      <c r="B38" s="23"/>
-      <c r="C38" s="23"/>
+      <c r="B38" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>231</v>
+      </c>
       <c r="D38" s="39"/>
       <c r="E38" s="39"/>
       <c r="F38" s="39"/>
       <c r="G38" s="39"/>
-      <c r="H38" s="39"/>
+      <c r="H38" s="39" t="n">
+        <v>1</v>
+      </c>
       <c r="I38" s="39"/>
       <c r="J38" s="39"/>
       <c r="K38" s="39"/>
-      <c r="L38" s="39"/>
+      <c r="L38" s="39" t="n">
+        <v>1</v>
+      </c>
       <c r="M38" s="39"/>
-      <c r="N38" s="23"/>
+      <c r="N38" s="23" t="n">
+        <v>0</v>
+      </c>
       <c r="O38" s="23"/>
       <c r="P38" s="23" t="n">
-        <v>12680</v>
-      </c>
-      <c r="Q38" s="40" t="n">
-        <v>11420</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q38" s="23"/>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="23"/>
@@ -6502,9 +7273,37 @@
       <c r="N39" s="23"/>
       <c r="O39" s="23"/>
       <c r="P39" s="23" t="n">
+        <v>12680</v>
+      </c>
+      <c r="Q39" s="42" t="n">
+        <v>11420</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="39"/>
+      <c r="E40" s="39"/>
+      <c r="F40" s="39"/>
+      <c r="G40" s="39"/>
+      <c r="H40" s="39"/>
+      <c r="I40" s="39"/>
+      <c r="J40" s="39"/>
+      <c r="K40" s="39"/>
+      <c r="L40" s="39"/>
+      <c r="M40" s="39"/>
+      <c r="N40" s="23"/>
+      <c r="O40" s="23"/>
+      <c r="P40" s="23" t="n">
         <v>1260</v>
       </c>
-      <c r="Q39" s="23"/>
+      <c r="Q40" s="23"/>
+    </row>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AH54" s="0" t="n">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>